<commit_message>
fixed some small issues and updated the colorscheme
</commit_message>
<xml_diff>
--- a/output/StructureDefinition-t-cabs-device-channel-beatmungsgeraet.xlsx
+++ b/output/StructureDefinition-t-cabs-device-channel-beatmungsgeraet.xlsx
@@ -27,7 +27,7 @@
     <t>URL</t>
   </si>
   <si>
-    <t>http://t-cabs.org/StructureDefinition/t-cabs-device-channel-beatmungsgeraet</t>
+    <t>https://bih-cei.github.io/T-CABS/StructureDefinition/t-cabs-device-channel-beatmungsgeraet</t>
   </si>
   <si>
     <t>Version</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-12-09T09:55:43+01:00</t>
+    <t>2026-02-19T13:21:58+01:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -1864,7 +1864,7 @@
     <t>Device.parent</t>
   </si>
   <si>
-    <t xml:space="preserve">Reference(http://t-cabs.org/StructureDefinition/t-cabs-device-vmd-beatmungsgeraet)
+    <t xml:space="preserve">Reference(https://bih-cei.github.io/T-CABS/StructureDefinition/t-cabs-device-vmd-beatmungsgeraet)
 </t>
   </si>
   <si>

</xml_diff>